<commit_message>
fix(import-preview): normalize imported fields and expand preview mapping
</commit_message>
<xml_diff>
--- a/test-data/xlsx/import_empty.xlsx
+++ b/test-data/xlsx/import_empty.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="import_empty" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -17,17 +17,6 @@
     </ext>
   </extLst>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
-  <si>
-    <t xml:space="preserve">Job Title</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Company</t>
-  </si>
-</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -227,22 +216,9 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8.39"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="9.14"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="0" t="s">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>